<commit_message>
Added some data files.
</commit_message>
<xml_diff>
--- a/additional_files/quality_check_filters.xlsx
+++ b/additional_files/quality_check_filters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\alex\alex_files\markerproject_redux\quality_check\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\alex\alex_files\markerproject_redux\scripts\additional_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE8202EE-B48C-4A3A-B575-AC1E44CE4ECF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A151469-C303-4AD8-B43F-28D07C9E085F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="15" xr2:uid="{B8D9EEE6-B46A-499B-AF53-BB0853FA40C2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="10" xr2:uid="{B8D9EEE6-B46A-499B-AF53-BB0853FA40C2}"/>
   </bookViews>
   <sheets>
     <sheet name="quality_check_filters" sheetId="1" r:id="rId1"/>
@@ -23,12 +23,11 @@
     <sheet name="Snf7" sheetId="8" r:id="rId8"/>
     <sheet name="Sec21" sheetId="9" r:id="rId9"/>
     <sheet name="Sec7" sheetId="10" r:id="rId10"/>
-    <sheet name="Psr1" sheetId="11" r:id="rId11"/>
-    <sheet name="Spf1" sheetId="12" r:id="rId12"/>
-    <sheet name="Om45" sheetId="13" r:id="rId13"/>
-    <sheet name="Heh2" sheetId="14" r:id="rId14"/>
-    <sheet name="Cdc11" sheetId="15" r:id="rId15"/>
-    <sheet name="Nop10" sheetId="16" r:id="rId16"/>
+    <sheet name="Spf1" sheetId="12" r:id="rId11"/>
+    <sheet name="Om45" sheetId="13" r:id="rId12"/>
+    <sheet name="Heh2" sheetId="14" r:id="rId13"/>
+    <sheet name="Cdc11" sheetId="15" r:id="rId14"/>
+    <sheet name="Nop10" sheetId="16" r:id="rId15"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -48,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1076" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1009" uniqueCount="121">
   <si>
     <t>Feature</t>
   </si>
@@ -366,12 +365,6 @@
   </si>
   <si>
     <t>&lt;=0.03</t>
-  </si>
-  <si>
-    <t>&gt;=2.3</t>
-  </si>
-  <si>
-    <t>&gt;=0.1</t>
   </si>
   <si>
     <t>&gt;=2.15</t>
@@ -1733,265 +1726,6 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{740F1600-2B79-467D-8B2B-493FF2967422}">
-  <dimension ref="A1:E23"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="40.140625" customWidth="1"/>
-    <col min="2" max="2" width="18.140625" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="E1" s="1"/>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D2" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" t="s">
-        <v>78</v>
-      </c>
-      <c r="D3" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4" t="s">
-        <v>46</v>
-      </c>
-      <c r="D4" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" t="s">
-        <v>85</v>
-      </c>
-      <c r="C5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D5" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" t="s">
-        <v>106</v>
-      </c>
-      <c r="D6" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" t="s">
-        <v>21</v>
-      </c>
-      <c r="C7" t="s">
-        <v>98</v>
-      </c>
-      <c r="D7" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" t="s">
-        <v>101</v>
-      </c>
-      <c r="D8" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>10</v>
-      </c>
-      <c r="C9" t="s">
-        <v>78</v>
-      </c>
-      <c r="D9" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>11</v>
-      </c>
-      <c r="B10" t="s">
-        <v>16</v>
-      </c>
-      <c r="C10" t="s">
-        <v>46</v>
-      </c>
-      <c r="D10" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B11" t="s">
-        <v>85</v>
-      </c>
-      <c r="C11" t="s">
-        <v>19</v>
-      </c>
-      <c r="D11" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" t="s">
-        <v>51</v>
-      </c>
-      <c r="C12" t="s">
-        <v>19</v>
-      </c>
-      <c r="D12" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>56</v>
-      </c>
-      <c r="C13" t="s">
-        <v>69</v>
-      </c>
-      <c r="D13" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>60</v>
-      </c>
-      <c r="C14" t="s">
-        <v>107</v>
-      </c>
-      <c r="D14" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>31</v>
-      </c>
-      <c r="B15" t="s">
-        <v>86</v>
-      </c>
-      <c r="D15" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>35</v>
-      </c>
-      <c r="B16" t="s">
-        <v>105</v>
-      </c>
-      <c r="C16" t="s">
-        <v>76</v>
-      </c>
-      <c r="D16" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>38</v>
-      </c>
-      <c r="B21" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>40</v>
-      </c>
-      <c r="B22" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>42</v>
-      </c>
-      <c r="B23" t="s">
-        <v>72</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7BE2379-53DD-4002-AA96-AC74473945C0}">
   <dimension ref="A1:E23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2077,7 +1811,7 @@
         <v>7</v>
       </c>
       <c r="C6" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="D6" t="s">
         <v>58</v>
@@ -2188,10 +1922,10 @@
         <v>31</v>
       </c>
       <c r="B15" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C15" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="D15" t="s">
         <v>59</v>
@@ -2250,7 +1984,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{015215E9-CE7B-4BCF-A558-C24442BB0A55}">
   <dimension ref="A1:E23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2336,7 +2070,7 @@
         <v>7</v>
       </c>
       <c r="C6" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D6" t="s">
         <v>58</v>
@@ -2361,7 +2095,7 @@
         <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="D8" t="s">
         <v>58</v>
@@ -2450,7 +2184,7 @@
         <v>32</v>
       </c>
       <c r="C15" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D15" t="s">
         <v>59</v>
@@ -2461,7 +2195,7 @@
         <v>35</v>
       </c>
       <c r="B16" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C16" t="s">
         <v>76</v>
@@ -2512,7 +2246,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D727EA25-5DBC-4F5C-812F-A4D22B9E0F46}">
   <dimension ref="A1:E23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2623,7 +2357,7 @@
         <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D8" t="s">
         <v>58</v>
@@ -2712,7 +2446,7 @@
         <v>32</v>
       </c>
       <c r="C15" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D15" t="s">
         <v>59</v>
@@ -2723,7 +2457,7 @@
         <v>35</v>
       </c>
       <c r="B16" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C16" t="s">
         <v>76</v>
@@ -2774,7 +2508,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37FAC35A-230C-4BD3-AB9C-0FD8AEEA84E6}">
   <dimension ref="A1:E23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2860,7 +2594,7 @@
         <v>7</v>
       </c>
       <c r="C6" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D6" t="s">
         <v>58</v>
@@ -3033,7 +2767,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F4DA24F-13B4-4F24-B0AB-A693783C1C64}">
   <dimension ref="A1:E23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3066,7 +2800,7 @@
         <v>16</v>
       </c>
       <c r="C2" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D2" t="s">
         <v>58</v>
@@ -3094,7 +2828,7 @@
         <v>16</v>
       </c>
       <c r="C4" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D4" t="s">
         <v>58</v>
@@ -3108,7 +2842,7 @@
         <v>87</v>
       </c>
       <c r="C5" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D5" t="s">
         <v>58</v>
@@ -3119,7 +2853,7 @@
         <v>7</v>
       </c>
       <c r="C6" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D6" t="s">
         <v>58</v>
@@ -3130,7 +2864,7 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C7" t="s">
         <v>80</v>
@@ -3144,7 +2878,7 @@
         <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D8" t="s">
         <v>58</v>
@@ -3172,7 +2906,7 @@
         <v>16</v>
       </c>
       <c r="C10" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D10" t="s">
         <v>58</v>
@@ -3186,7 +2920,7 @@
         <v>87</v>
       </c>
       <c r="C11" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D11" t="s">
         <v>58</v>
@@ -3247,7 +2981,7 @@
         <v>35</v>
       </c>
       <c r="B16" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C16" t="s">
         <v>76</v>

</xml_diff>